<commit_message>
Fix data import and other issues
</commit_message>
<xml_diff>
--- a/TestExpenditure.xlsx
+++ b/TestExpenditure.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manuv\Documents\Code\PyPrograms\Budget-Tracker\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mmohan\source\repos\Budget-Tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FADE8DD9-C31A-4F9C-8BE1-F621AB7C2E8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{760F1046-CA8F-4060-9BD6-CB0165C2AE73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38510" yWindow="-7540" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38510" yWindow="-6490" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -93,40 +93,40 @@
     <t>General</t>
   </si>
   <si>
-    <t>Jan-23</t>
-  </si>
-  <si>
-    <t>Feb-23</t>
-  </si>
-  <si>
-    <t>Mar-23</t>
-  </si>
-  <si>
-    <t>Apr-23</t>
-  </si>
-  <si>
-    <t>May-23</t>
-  </si>
-  <si>
-    <t>Jun-23</t>
-  </si>
-  <si>
-    <t>Jul-23</t>
-  </si>
-  <si>
-    <t>Aug-23</t>
-  </si>
-  <si>
-    <t>Sep-23</t>
-  </si>
-  <si>
-    <t>Oct-23</t>
-  </si>
-  <si>
-    <t>Nov-23</t>
-  </si>
-  <si>
-    <t>Dec-23</t>
+    <t>Jan-22</t>
+  </si>
+  <si>
+    <t>Feb-22</t>
+  </si>
+  <si>
+    <t>Mar-22</t>
+  </si>
+  <si>
+    <t>Apr-22</t>
+  </si>
+  <si>
+    <t>May-22</t>
+  </si>
+  <si>
+    <t>Jun-22</t>
+  </si>
+  <si>
+    <t>Aug-22</t>
+  </si>
+  <si>
+    <t>Sep-22</t>
+  </si>
+  <si>
+    <t>Oct-22</t>
+  </si>
+  <si>
+    <t>Nov-22</t>
+  </si>
+  <si>
+    <t>Dec-22</t>
+  </si>
+  <si>
+    <t>Jul-22</t>
   </si>
 </sst>
 </file>
@@ -136,7 +136,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$$-1409]#,##0.00"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -162,6 +162,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -259,914 +265,884 @@
     <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="94">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
+  <dxfs count="91">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1505,22 +1481,22 @@
         <v>27</v>
       </c>
       <c r="H1" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I1" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="J1" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="J1" s="7" t="s">
+      <c r="K1" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="K1" s="7" t="s">
+      <c r="L1" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="L1" s="7" t="s">
+      <c r="M1" s="7" t="s">
         <v>32</v>
-      </c>
-      <c r="M1" s="7" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -2358,28 +2334,18 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="B2:B23 C2:M2">
-    <cfRule type="cellIs" dxfId="93" priority="94" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="90" priority="94" operator="greaterThan">
       <formula>$B$2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B8:B10">
-    <cfRule type="cellIs" dxfId="92" priority="82" operator="lessThan">
+    <cfRule type="cellIs" dxfId="89" priority="82" operator="lessThan">
       <formula>$B$8</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="91" priority="83" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="88" priority="83" operator="greaterThan">
       <formula>$B$8</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:M2">
-    <cfRule type="cellIs" dxfId="89" priority="64" operator="lessThan">
-      <formula>$B$2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="88" priority="65" operator="greaterThan">
-      <formula>$B$2</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="90" priority="87" operator="lessThan">
-      <formula>$B$2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:C3">
@@ -2391,10 +2357,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B4:C4">
-    <cfRule type="cellIs" dxfId="85" priority="88" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="85" priority="92" operator="greaterThan">
       <formula>$B$4</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="84" priority="92" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="84" priority="88" operator="greaterThan">
       <formula>$B$4</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2420,19 +2386,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B10:C10">
+    <cfRule type="cellIs" dxfId="78" priority="81" operator="greaterThan">
+      <formula>$B$10</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="77" priority="80" operator="lessThan">
       <formula>$B$10</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="78" priority="81" operator="greaterThan">
-      <formula>$B$10</formula>
-    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B11:C11">
+    <cfRule type="cellIs" dxfId="76" priority="79" operator="greaterThan">
+      <formula>-1465.62</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="75" priority="78" operator="greaterThan">
       <formula>$B$11</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="76" priority="79" operator="greaterThan">
-      <formula>-1465.62</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B12:C12">
@@ -2585,114 +2551,125 @@
       <formula>$B$6</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B2:M2">
+    <cfRule type="cellIs" dxfId="44" priority="87" operator="lessThan">
+      <formula>$B$2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="43" priority="64" operator="lessThan">
+      <formula>$B$2</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="42" priority="65" operator="greaterThan">
+      <formula>$B$2</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C3:C23">
-    <cfRule type="cellIs" dxfId="44" priority="63" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="41" priority="63" operator="greaterThan">
       <formula>$B$2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C8:C10">
-    <cfRule type="cellIs" dxfId="42" priority="61" operator="lessThan">
+    <cfRule type="cellIs" dxfId="40" priority="62" operator="greaterThan">
       <formula>$B$8</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="43" priority="62" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="39" priority="61" operator="lessThan">
       <formula>$B$8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C23">
-    <cfRule type="cellIs" dxfId="41" priority="60" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="38" priority="60" operator="greaterThan">
       <formula>$B$2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10:D10">
-    <cfRule type="cellIs" dxfId="38" priority="39" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="37" priority="39" operator="greaterThan">
       <formula>$B$10</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="39" priority="52" operator="lessThan">
+    <cfRule type="cellIs" dxfId="36" priority="52" operator="lessThan">
       <formula>$B$10</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C23:D23">
-    <cfRule type="cellIs" dxfId="37" priority="28" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="35" priority="28" operator="greaterThan">
       <formula>$B$23</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D8">
-    <cfRule type="cellIs" dxfId="35" priority="54" operator="lessThan">
+    <cfRule type="cellIs" dxfId="34" priority="54" operator="lessThan">
       <formula>$B$8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9">
-    <cfRule type="cellIs" dxfId="34" priority="53" operator="lessThan">
+    <cfRule type="cellIs" dxfId="33" priority="53" operator="lessThan">
       <formula>$B$9</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D11">
-    <cfRule type="cellIs" dxfId="33" priority="38" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="32" priority="38" operator="greaterThan">
       <formula>$B$11</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D13">
-    <cfRule type="cellIs" dxfId="32" priority="37" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="31" priority="37" operator="greaterThan">
       <formula>$B$13</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D14">
-    <cfRule type="cellIs" dxfId="31" priority="36" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="30" priority="36" operator="greaterThan">
       <formula>$B$14</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D15">
-    <cfRule type="cellIs" dxfId="30" priority="35" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="29" priority="35" operator="greaterThan">
       <formula>$B$15</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D17">
-    <cfRule type="cellIs" dxfId="29" priority="34" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="28" priority="34" operator="greaterThan">
       <formula>$B$17</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D18">
-    <cfRule type="cellIs" dxfId="28" priority="33" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="27" priority="33" operator="greaterThan">
       <formula>$B$18</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D19">
-    <cfRule type="cellIs" dxfId="27" priority="32" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="26" priority="32" operator="greaterThan">
       <formula>$B$19</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D20">
-    <cfRule type="cellIs" dxfId="26" priority="31" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="25" priority="31" operator="greaterThan">
       <formula>$B$20</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D21">
-    <cfRule type="cellIs" dxfId="25" priority="30" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="24" priority="30" operator="greaterThan">
       <formula>$B$21</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D22">
-    <cfRule type="cellIs" dxfId="24" priority="29" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="23" priority="29" operator="greaterThan">
       <formula>$B$22</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:E7">
-    <cfRule type="cellIs" dxfId="23" priority="23" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="22" priority="23" operator="greaterThan">
       <formula>$B$7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D9:E9">
-    <cfRule type="cellIs" dxfId="22" priority="20" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="21" priority="20" operator="greaterThan">
       <formula>$B$9</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D12:E12">
-    <cfRule type="cellIs" dxfId="21" priority="17" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="20" priority="17" operator="greaterThan">
       <formula>$B$12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D16:E16">
-    <cfRule type="cellIs" dxfId="20" priority="12" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="19" priority="12" operator="greaterThan">
       <formula>$B$16</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2777,10 +2754,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6:F6">
+    <cfRule type="cellIs" dxfId="2" priority="24" operator="greaterThan">
+      <formula>$B$6</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="1" priority="6" operator="lessThan">
-      <formula>$B$6</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="24" operator="greaterThan">
       <formula>$B$6</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2790,5 +2767,14 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter>
+    <oddFooter>&amp;L_x000D_&amp;1#&amp;"Calibri"&amp;8&amp;K000000 Classification: Private</oddFooter>
+  </headerFooter>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{7b044127-70a7-491f-af80-ec53910828db}" enabled="1" method="Standard" siteId="{90db3e97-44ee-44d6-a14c-518e66b35785}" contentBits="2" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>